<commit_message>
Maliyet dokümanı ve fiyat modeline TTS karşılaştırması
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gbsoft-fiyat-modeli.xlsx
+++ b/gbsoft-fiyat-modeli.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ozet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geliştirme_Araclari" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sunucu_Barindirma" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Uretim" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24_Ay_Senaryo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sozlesme_Maddeleri" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canli_AltYapi" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Ozet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Geliştirme_Araclari" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sunucu_Barindirma" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="AI_Uretim" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="24_Ay_Senaryo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sozlesme_Maddeleri" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Canli_AltYapi" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -22,10 +22,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="166" formatCode="#,##0&quot; TL&quot;;\(#,##0&quot;) TL&quot;;\-"/>
+    <numFmt numFmtId="167" formatCode="$0.000"/>
+    <numFmt numFmtId="168" formatCode="$#,##0"/>
+    <numFmt numFmtId="169" formatCode="€#,##0"/>
+    <numFmt numFmtId="170" formatCode="$0.00"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -287,7 +291,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -450,6 +454,30 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -729,7 +757,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="27">
       <c r="A4" s="30" t="inlineStr">
         <is>
@@ -803,7 +830,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="15" customHeight="1" s="27">
       <c r="A10" s="30" t="inlineStr">
         <is>
@@ -897,7 +923,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="27">
       <c r="A16" s="26" t="inlineStr">
         <is>
@@ -918,7 +943,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="15" customHeight="1" s="27">
       <c r="A18" s="43" t="inlineStr">
         <is>
@@ -979,7 +1003,6 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="15" customHeight="1" s="27">
       <c r="A24" s="30" t="inlineStr">
         <is>
@@ -1104,7 +1127,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30" ht="15" customHeight="1" s="27">
       <c r="A30" s="30" t="inlineStr">
         <is>
@@ -2568,12 +2590,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="26" min="1" max="1"/>
     <col width="22" customWidth="1" style="26" min="2" max="4"/>
+    <col width="14" customWidth="1" style="27" min="3" max="3"/>
+    <col width="16" customWidth="1" style="27" min="4" max="4"/>
     <col width="14" customWidth="1" style="26" min="5" max="6"/>
+    <col width="18" customWidth="1" style="27" min="6" max="6"/>
+    <col width="60" customWidth="1" style="27" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" s="27">
@@ -2688,7 +2714,7 @@
       </c>
       <c r="C10" s="29" t="inlineStr">
         <is>
-          <t>openai.com/api/pricing — TTS $15/1M karakter (Std); dakika başına tahmini yaklaşım</t>
+          <t>gpt-4o-mini-tts ≈ $0.015/dk (tahmini); alternatifler için aşağıdaki TTS tablosu</t>
         </is>
       </c>
     </row>
@@ -2982,6 +3008,318 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="43" t="inlineStr">
+        <is>
+          <t>TTS MODEL KARŞILAŞTIRMASI (fiyat kontrolü: Ekim 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="47" t="inlineStr">
+        <is>
+          <t>Dakika başına karakter (tahmin)</t>
+        </is>
+      </c>
+      <c r="B36" s="33" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C36" s="29" t="inlineStr">
+        <is>
+          <t>Türkçe konuşma ≈ 900–1.000 karakter/dk</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="47" t="inlineStr">
+        <is>
+          <t>Sesi açan misafir oranı</t>
+        </is>
+      </c>
+      <c r="B37" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="29" t="inlineStr">
+        <is>
+          <t>1 = tavan senaryo; gerçekçi tahmin için 0,3 dene</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
+    <row r="39">
+      <c r="A39" s="49" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B39" s="49" t="inlineStr">
+        <is>
+          <t>USD / 1M karakter</t>
+        </is>
+      </c>
+      <c r="C39" s="49" t="inlineStr">
+        <is>
+          <t>USD / dakika</t>
+        </is>
+      </c>
+      <c r="D39" s="49" t="inlineStr">
+        <is>
+          <t>Tur başı (USD)</t>
+        </is>
+      </c>
+      <c r="E39" s="49" t="inlineStr">
+        <is>
+          <t>Otel başı / ay (USD)</t>
+        </is>
+      </c>
+      <c r="F39" s="49" t="inlineStr">
+        <is>
+          <t>Platform / ay (USD)</t>
+        </is>
+      </c>
+      <c r="G39" s="49" t="inlineStr">
+        <is>
+          <t>Not / kaynak</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="47" t="inlineStr">
+        <is>
+          <t>OpenAI gpt-4o-mini-tts (sohbet — öneri)</t>
+        </is>
+      </c>
+      <c r="C40" s="61" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="D40" s="62">
+        <f>C40*$B$8*$B$37</f>
+        <v/>
+      </c>
+      <c r="E40" s="51">
+        <f>D40*$B$15</f>
+        <v/>
+      </c>
+      <c r="F40" s="51">
+        <f>E40*Ozet!$B$8</f>
+        <v/>
+      </c>
+      <c r="G40" s="29" t="inlineStr">
+        <is>
+          <t>Token bazlı; ~$0.015/dk üçüncü taraf kaynak — resmi sayfadan teyit et</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="47" t="inlineStr">
+        <is>
+          <t>Azure Neural TTS</t>
+        </is>
+      </c>
+      <c r="B41" s="63" t="n">
+        <v>15</v>
+      </c>
+      <c r="C41" s="62">
+        <f>B41*$B$36/1000000</f>
+        <v/>
+      </c>
+      <c r="D41" s="62">
+        <f>C41*$B$8*$B$37</f>
+        <v/>
+      </c>
+      <c r="E41" s="51">
+        <f>D41*$B$15</f>
+        <v/>
+      </c>
+      <c r="F41" s="51">
+        <f>E41*Ozet!$B$8</f>
+        <v/>
+      </c>
+      <c r="G41" s="29" t="inlineStr">
+        <is>
+          <t>tr-TR sesleri var; üçüncü taraf kaynak — teyit et</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="47" t="inlineStr">
+        <is>
+          <t>Google Chirp 3 HD</t>
+        </is>
+      </c>
+      <c r="B42" s="63" t="n">
+        <v>30</v>
+      </c>
+      <c r="C42" s="62">
+        <f>B42*$B$36/1000000</f>
+        <v/>
+      </c>
+      <c r="D42" s="62">
+        <f>C42*$B$8*$B$37</f>
+        <v/>
+      </c>
+      <c r="E42" s="51">
+        <f>D42*$B$15</f>
+        <v/>
+      </c>
+      <c r="F42" s="51">
+        <f>E42*Ozet!$B$8</f>
+        <v/>
+      </c>
+      <c r="G42" s="29" t="inlineStr">
+        <is>
+          <t>cloud.google.com/text-to-speech/pricing — ilk 1M karakter/ay ücretsiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="47" t="inlineStr">
+        <is>
+          <t>ElevenLabs Flash/Turbo</t>
+        </is>
+      </c>
+      <c r="B43" s="63" t="n">
+        <v>40</v>
+      </c>
+      <c r="C43" s="62">
+        <f>B43*$B$36/1000000</f>
+        <v/>
+      </c>
+      <c r="D43" s="62">
+        <f>C43*$B$8*$B$37</f>
+        <v/>
+      </c>
+      <c r="E43" s="51">
+        <f>D43*$B$15</f>
+        <v/>
+      </c>
+      <c r="F43" s="51">
+        <f>E43*Ozet!$B$8</f>
+        <v/>
+      </c>
+      <c r="G43" s="29" t="inlineStr">
+        <is>
+          <t>elevenlabs.io/pricing/api — $0.04/1K; abonelik paketi düşürür</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="47" t="inlineStr">
+        <is>
+          <t>ElevenLabs v3 / Multilingual v2 (anlatım — öneri)</t>
+        </is>
+      </c>
+      <c r="B44" s="63" t="n">
+        <v>80</v>
+      </c>
+      <c r="C44" s="62">
+        <f>B44*$B$36/1000000</f>
+        <v/>
+      </c>
+      <c r="D44" s="62">
+        <f>C44*$B$8*$B$37</f>
+        <v/>
+      </c>
+      <c r="E44" s="51">
+        <f>D44*$B$15</f>
+        <v/>
+      </c>
+      <c r="F44" s="51">
+        <f>E44*Ozet!$B$8</f>
+        <v/>
+      </c>
+      <c r="G44" s="29" t="inlineStr">
+        <is>
+          <t>elevenlabs.io/pricing/api — $0.08/1K; sabit anlatım için</t>
+        </is>
+      </c>
+    </row>
+    <row r="45"/>
+    <row r="46">
+      <c r="A46" s="43" t="inlineStr">
+        <is>
+          <t>ADIM ANLATIMI ÖN ÜRETİM (tek seferlik, otel başı)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="47" t="inlineStr">
+        <is>
+          <t>Otel başı anlatım karakteri (tüm adımlar × diller)</t>
+        </is>
+      </c>
+      <c r="B47" s="33" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C47" s="29" t="inlineStr">
+        <is>
+          <t>Tahmin: ~10 adım × 500 karakter × 2 dil; bir kez üretilip R2'de saklanır</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="64" t="inlineStr">
+        <is>
+          <t>Tek seferlik maliyet (ElevenLabs v3, USD)</t>
+        </is>
+      </c>
+      <c r="B48" s="65">
+        <f>B47/1000000*B44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="43" t="inlineStr">
+        <is>
+          <t>KENDİ GPU ALTERNATİFİ (API yerine)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="47" t="inlineStr">
+        <is>
+          <t>Hetzner GEX44 (RTX 4000 Ada) — EUR/ay, GPU başı</t>
+        </is>
+      </c>
+      <c r="B51" s="66" t="n">
+        <v>184</v>
+      </c>
+      <c r="C51" s="29" t="inlineStr">
+        <is>
+          <t>+ €79 kurulum. Model: Chatterbox Multilingual (MIT, Türkçe var)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="47" t="inlineStr">
+        <is>
+          <t>RunPod RTX 4090 — USD/saat</t>
+        </is>
+      </c>
+      <c r="B52" s="67" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C52" s="29" t="inlineStr">
+        <is>
+          <t>Sürekli açık ≈ $440/ay; fiyat üçüncü taraf kaynak</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="47" t="inlineStr">
+        <is>
+          <t>Not</t>
+        </is>
+      </c>
+      <c r="C53" s="29" t="inlineStr">
+        <is>
+          <t>GPU sayısı ve Türkçe kalite ölçülmedi; ~40.000 dk/ay altında API daha ucuz (tahmin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54"/>
+    <row r="55"/>
   </sheetData>
   <mergeCells count="19">
     <mergeCell ref="C8:F8"/>

</xml_diff>